<commit_message>
Ledgr: update my-money.xlsx (2026-08-22T20:45:09.370Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -6081,7 +6081,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6139,9 +6139,17 @@
         <v>No</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Advanced</v>
+      </c>
+      <c r="B8" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ledgr: update my-money.xlsx (2026-10-08T06:48:41.999Z)
</commit_message>
<xml_diff>
--- a/my-money.xlsx
+++ b/my-money.xlsx
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2088,9 +2088,56 @@
         <v>EVT-01</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TXN-10035</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-10-08</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Income</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Debt Settlement</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Repayment received from Albert</v>
+      </c>
+      <c r="G38">
+        <v>78700</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Federal-Ang</v>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v>Auto-Posted: DEBT-01 (Albert)</v>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2294,13 +2341,13 @@
         <v>28000</v>
       </c>
       <c r="F6">
-        <v>42000</v>
+        <v>120700</v>
       </c>
       <c r="G6">
         <v>161050</v>
       </c>
       <c r="H6">
-        <v>-91050</v>
+        <v>-12350</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -2665,10 +2712,10 @@
         <v>78700</v>
       </c>
       <c r="J4">
+        <v>78700</v>
+      </c>
+      <c r="K4">
         <v>0</v>
-      </c>
-      <c r="K4">
-        <v>78700</v>
       </c>
       <c r="L4" t="str">
         <v>2026-05-10</v>
@@ -2677,16 +2724,16 @@
         <v>2026-09-22</v>
       </c>
       <c r="N4" t="str">
-        <v>Open</v>
+        <v>Closed</v>
       </c>
       <c r="O4" t="str">
-        <v/>
+        <v>2026-10-08</v>
       </c>
       <c r="P4" t="str">
-        <v/>
+        <v>Federal-Ang</v>
       </c>
       <c r="Q4" t="str">
-        <v/>
+        <v>TXN-10035</v>
       </c>
       <c r="R4" t="str">
         <v>13001</v>
@@ -6156,7 +6203,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7512,16 +7559,54 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TXN-10035</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-10-08</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Income</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Income</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Repayment received from Albert · Auto-Posted: DEBT-01 (Albert)</v>
+      </c>
+      <c r="F38">
+        <v>78700</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v>Auto-Posted: DEBT-01 (Albert)</v>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38">
+        <v>2</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L38"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L75"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -10245,16 +10330,92 @@
         <v>ACC-02</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>TXN-10035-L1</v>
+      </c>
+      <c r="B74" t="str">
+        <v>TXN-10035</v>
+      </c>
+      <c r="C74">
+        <v>1</v>
+      </c>
+      <c r="D74">
+        <v>78700</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="F74" t="str">
+        <v>11003</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Federal-Ang Bank</v>
+      </c>
+      <c r="H74" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I74" t="str">
+        <v>Cash &amp; Bank</v>
+      </c>
+      <c r="J74" t="str">
+        <v>Debit</v>
+      </c>
+      <c r="K74" t="str">
+        <v>Bank</v>
+      </c>
+      <c r="L74" t="str">
+        <v>ACC-03</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>TXN-10035-L2</v>
+      </c>
+      <c r="B75" t="str">
+        <v>TXN-10035</v>
+      </c>
+      <c r="C75">
+        <v>2</v>
+      </c>
+      <c r="D75">
+        <v>-78700</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="F75" t="str">
+        <v>13001</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Loans Given (Receivables)</v>
+      </c>
+      <c r="H75" t="str">
+        <v>Asset</v>
+      </c>
+      <c r="I75" t="str">
+        <v>Receivables</v>
+      </c>
+      <c r="J75" t="str">
+        <v>Credit</v>
+      </c>
+      <c r="K75" t="str">
+        <v>Loan</v>
+      </c>
+      <c r="L75" t="str">
+        <v>DEBT-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L75"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11176,9 +11337,38 @@
         <v>Test</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TXN-10035-L1</v>
+      </c>
+      <c r="B34" t="str">
+        <v>ACC-03</v>
+      </c>
+      <c r="C34" t="str">
+        <v>TXN-10035</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2026-10-08</v>
+      </c>
+      <c r="F34">
+        <v>78700</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Dr</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Federal-Ang Bank</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Repayment received from Albert · Auto-Posted: DEBT-01 (Albert)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11420,7 +11610,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11559,9 +11749,38 @@
         <v>Bought gadget - split with Baby</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TXN-10035-L2</v>
+      </c>
+      <c r="B7" t="str">
+        <v>DEBT-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>TXN-10035</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-10-08</v>
+      </c>
+      <c r="F7">
+        <v>-78700</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Cr</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Loans Given (Receivables)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Repayment received from Albert · Auto-Posted: DEBT-01 (Albert)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>